<commit_message>
with layer css js
</commit_message>
<xml_diff>
--- a/Excel Files/OS.xlsx
+++ b/Excel Files/OS.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub projects\Mcq_generator\Excel Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD63D7C0-302F-46F2-8459-307488ED83C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE29824-B2EF-4604-B29D-92889CD84D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A7744768-14E7-4F39-B6A5-4D54AC18E601}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="252">
   <si>
     <t>1 Mark</t>
   </si>
@@ -706,6 +707,129 @@
   </si>
   <si>
     <t>True: FIFO is not a disk scheduling algorithm.</t>
+  </si>
+  <si>
+    <t>Question text</t>
+  </si>
+  <si>
+    <t>Question type</t>
+  </si>
+  <si>
+    <t>Answer (mcq &amp; TF)/
+marks (single)</t>
+  </si>
+  <si>
+    <t>Option B/ 2 marks</t>
+  </si>
+  <si>
+    <t>Option C/ 3 marks</t>
+  </si>
+  <si>
+    <t>Option D/4 marks</t>
+  </si>
+  <si>
+    <t>Option E / 5 marks</t>
+  </si>
+  <si>
+    <t>Option F / 6 marks</t>
+  </si>
+  <si>
+    <t>Option G / 7 marks</t>
+  </si>
+  <si>
+    <t>Written Single</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>The kernel manages hardware resources.</t>
+  </si>
+  <si>
+    <t>True/False</t>
+  </si>
+  <si>
+    <t>FCFS always minimizes average waiting time.</t>
+  </si>
+  <si>
+    <t>Paging avoids external fragmentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Compilation is a system call.</t>
+  </si>
+  <si>
+    <t>Banker’s algorithm ensures safe state.</t>
+  </si>
+  <si>
+    <t>Round Robin is non-preemptive.</t>
+  </si>
+  <si>
+    <t>LOOK is a disk scheduling algorithm.</t>
+  </si>
+  <si>
+    <t>Threads reduce memory usage.</t>
+  </si>
+  <si>
+    <t>Semaphores prevent race conditions.</t>
+  </si>
+  <si>
+    <t>Logical fragmentation exists in OS.</t>
+  </si>
+  <si>
+    <t>All listed are page replacement algorithms.</t>
+  </si>
+  <si>
+    <t>OS directly manages browsing.</t>
+  </si>
+  <si>
+    <t>All are IPC mechanisms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Compilation speed is a criterion.</t>
+  </si>
+  <si>
+    <t>Both hard and soft RTOS exist.</t>
+  </si>
+  <si>
+    <t>Random allocation is valid.</t>
+  </si>
+  <si>
+    <t>All four are deadlock conditions.</t>
+  </si>
+  <si>
+    <t>All are valid scheduling queues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Fast Fit is a strategy.</t>
+  </si>
+  <si>
+    <t>FIFO is not a disk scheduling algorithm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A disk drive has 5000 cylinders. Current head at 143, previous at 125. Queue: 86, 1470, 913, 1774, 948, 1509, 1022, 1750, 130.</t>
+  </si>
+  <si>
+    <t>Written
+Layered</t>
+  </si>
+  <si>
+    <t>Resource allocation graph with processes P1, P2, P3 and resources R1, R2, R3.</t>
+  </si>
+  <si>
+    <t>Processes with burst times and priorities (P1=2, P2=1, P3=8, P4=4, P5=5).</t>
+  </si>
+  <si>
+    <t>Define burst time and waiting time of a process.</t>
+  </si>
+  <si>
+    <t>Explain an advantage of FCFS over SJF.</t>
+  </si>
+  <si>
+    <t>Option A (MCQ)/ 
+1 mark (layered)</t>
+  </si>
+  <si>
+    <t>Explain Priority Based scheduling for this table.</t>
   </si>
 </sst>
 </file>
@@ -749,7 +873,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -759,6 +883,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,6 +1215,2327 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3EF6645-2ADC-41FF-AEBE-A7F498CAD0CF}">
+  <dimension ref="A1:J115"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.77734375" customWidth="1"/>
+    <col min="2" max="10" width="23.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C2" s="7">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="J2" s="7"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C3" s="7">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="J3" s="7"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C4" s="7">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" s="7">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="7">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C7" s="7">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C8" s="7">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C9" s="7">
+        <v>1</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C10" s="7">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C11" s="7">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C12" s="7">
+        <v>2</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C13" s="7">
+        <v>2</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C14" s="7">
+        <v>2</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+    </row>
+    <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C15" s="7">
+        <v>2</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C16" s="7">
+        <v>2</v>
+      </c>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+    </row>
+    <row r="17" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C17" s="7">
+        <v>2</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+    </row>
+    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C18" s="7">
+        <v>2</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C19" s="7">
+        <v>2</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+    </row>
+    <row r="20" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C20" s="7">
+        <v>2</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+    </row>
+    <row r="21" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C21" s="7">
+        <v>2</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+    </row>
+    <row r="22" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C22" s="7">
+        <v>3</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+    </row>
+    <row r="23" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C23" s="7">
+        <v>3</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+    </row>
+    <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" s="7">
+        <v>3</v>
+      </c>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+    </row>
+    <row r="25" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C25" s="7">
+        <v>3</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+    </row>
+    <row r="26" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C26" s="7">
+        <v>3</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+    </row>
+    <row r="27" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C27" s="7">
+        <v>3</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+    </row>
+    <row r="28" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C28" s="7">
+        <v>3</v>
+      </c>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+    </row>
+    <row r="29" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C29" s="7">
+        <v>3</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+    </row>
+    <row r="30" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C30" s="7">
+        <v>3</v>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="7"/>
+    </row>
+    <row r="31" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C31" s="7">
+        <v>3</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+    </row>
+    <row r="32" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C32" s="7">
+        <v>4</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+    </row>
+    <row r="33" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C33" s="7">
+        <v>4</v>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+    </row>
+    <row r="34" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C34" s="7">
+        <v>4</v>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C35" s="7">
+        <v>4</v>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+    </row>
+    <row r="36" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C36" s="7">
+        <v>4</v>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="7"/>
+    </row>
+    <row r="37" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C37" s="7">
+        <v>4</v>
+      </c>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
+    </row>
+    <row r="38" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C38" s="7">
+        <v>4</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="7"/>
+    </row>
+    <row r="39" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C39" s="7">
+        <v>4</v>
+      </c>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="7"/>
+    </row>
+    <row r="40" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C40" s="7">
+        <v>4</v>
+      </c>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+    </row>
+    <row r="41" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C41" s="7">
+        <v>4</v>
+      </c>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="7"/>
+    </row>
+    <row r="42" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C42" s="7">
+        <v>5</v>
+      </c>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="7"/>
+    </row>
+    <row r="43" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C43" s="7">
+        <v>5</v>
+      </c>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7"/>
+    </row>
+    <row r="44" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C44" s="7">
+        <v>5</v>
+      </c>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="7"/>
+      <c r="J44" s="7"/>
+    </row>
+    <row r="45" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C45" s="7">
+        <v>5</v>
+      </c>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+    </row>
+    <row r="46" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C46" s="7">
+        <v>5</v>
+      </c>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="7"/>
+    </row>
+    <row r="47" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C47" s="7">
+        <v>5</v>
+      </c>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="7"/>
+      <c r="J47" s="7"/>
+    </row>
+    <row r="48" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C48" s="7">
+        <v>5</v>
+      </c>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7"/>
+    </row>
+    <row r="49" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C49" s="7">
+        <v>5</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+    </row>
+    <row r="50" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C50" s="7">
+        <v>5</v>
+      </c>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
+    </row>
+    <row r="51" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C51" s="7">
+        <v>5</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+    </row>
+    <row r="52" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C52" s="7">
+        <v>6</v>
+      </c>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
+      <c r="J52" s="7"/>
+    </row>
+    <row r="53" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C53" s="7">
+        <v>6</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+    </row>
+    <row r="54" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C54" s="7">
+        <v>6</v>
+      </c>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+    </row>
+    <row r="55" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C55" s="7">
+        <v>6</v>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+    </row>
+    <row r="56" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C56" s="7">
+        <v>6</v>
+      </c>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="7"/>
+    </row>
+    <row r="57" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C57" s="7">
+        <v>6</v>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+    </row>
+    <row r="58" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C58" s="7">
+        <v>6</v>
+      </c>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="7"/>
+    </row>
+    <row r="59" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C59" s="7">
+        <v>6</v>
+      </c>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+    </row>
+    <row r="60" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A60" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C60" s="7">
+        <v>6</v>
+      </c>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+      <c r="J60" s="7"/>
+    </row>
+    <row r="61" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C61" s="7">
+        <v>6</v>
+      </c>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+    </row>
+    <row r="62" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A62" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C62" s="7">
+        <v>7</v>
+      </c>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+      <c r="J62" s="7"/>
+    </row>
+    <row r="63" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C63" s="7">
+        <v>7</v>
+      </c>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+    </row>
+    <row r="64" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A64" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C64" s="7">
+        <v>7</v>
+      </c>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
+      <c r="I64" s="7"/>
+      <c r="J64" s="7"/>
+    </row>
+    <row r="65" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C65" s="7">
+        <v>7</v>
+      </c>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="7"/>
+      <c r="I65" s="7"/>
+      <c r="J65" s="7"/>
+    </row>
+    <row r="66" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A66" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C66" s="7">
+        <v>7</v>
+      </c>
+      <c r="D66" s="7"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7"/>
+      <c r="G66" s="7"/>
+      <c r="H66" s="7"/>
+      <c r="I66" s="7"/>
+      <c r="J66" s="7"/>
+    </row>
+    <row r="67" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C67" s="7">
+        <v>7</v>
+      </c>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+    </row>
+    <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C68" s="7">
+        <v>7</v>
+      </c>
+      <c r="D68" s="7"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="7"/>
+      <c r="I68" s="7"/>
+      <c r="J68" s="7"/>
+    </row>
+    <row r="69" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C69" s="7">
+        <v>7</v>
+      </c>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="7"/>
+      <c r="I69" s="7"/>
+      <c r="J69" s="7"/>
+    </row>
+    <row r="70" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C70" s="7">
+        <v>7</v>
+      </c>
+      <c r="D70" s="7"/>
+      <c r="E70" s="7"/>
+      <c r="F70" s="7"/>
+      <c r="G70" s="7"/>
+      <c r="H70" s="7"/>
+      <c r="I70" s="7"/>
+      <c r="J70" s="7"/>
+    </row>
+    <row r="71" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C71" s="7">
+        <v>7</v>
+      </c>
+      <c r="D71" s="7"/>
+      <c r="E71" s="7"/>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="7"/>
+      <c r="I71" s="7"/>
+      <c r="J71" s="7"/>
+    </row>
+    <row r="72" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A72" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E72" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G72" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H72" s="7"/>
+      <c r="I72" s="7"/>
+      <c r="J72" s="7"/>
+    </row>
+    <row r="73" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A73" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F73" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G73" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="H73" s="7"/>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+    </row>
+    <row r="74" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A74" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="G74" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H74" s="7"/>
+      <c r="I74" s="7"/>
+      <c r="J74" s="7"/>
+    </row>
+    <row r="75" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="F75" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G75" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="H75" s="7"/>
+      <c r="I75" s="7"/>
+      <c r="J75" s="7"/>
+    </row>
+    <row r="76" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E76" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F76" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="H76" s="7"/>
+      <c r="I76" s="7"/>
+      <c r="J76" s="7"/>
+    </row>
+    <row r="77" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A77" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F77" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H77" s="7"/>
+      <c r="I77" s="7"/>
+      <c r="J77" s="7"/>
+    </row>
+    <row r="78" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A78" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F78" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="H78" s="7"/>
+      <c r="I78" s="7"/>
+      <c r="J78" s="7"/>
+    </row>
+    <row r="79" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A79" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F79" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H79" s="7"/>
+      <c r="I79" s="7"/>
+      <c r="J79" s="7"/>
+    </row>
+    <row r="80" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E80" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="F80" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="G80" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="H80" s="7"/>
+      <c r="I80" s="7"/>
+      <c r="J80" s="7"/>
+    </row>
+    <row r="81" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A81" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D81" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="F81" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="G81" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H81" s="7"/>
+      <c r="I81" s="7"/>
+      <c r="J81" s="7"/>
+    </row>
+    <row r="82" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B82" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D82" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="E82" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="F82" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="G82" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="H82" s="7"/>
+      <c r="I82" s="7"/>
+      <c r="J82" s="7"/>
+    </row>
+    <row r="83" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A83" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D83" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E83" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="F83" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="G83" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="H83" s="7"/>
+      <c r="I83" s="7"/>
+      <c r="J83" s="7"/>
+    </row>
+    <row r="84" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A84" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D84" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E84" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="G84" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="H84" s="7"/>
+      <c r="I84" s="7"/>
+      <c r="J84" s="7"/>
+    </row>
+    <row r="85" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A85" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B85" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E85" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F85" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="G85" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="H85" s="7"/>
+      <c r="I85" s="7"/>
+      <c r="J85" s="7"/>
+    </row>
+    <row r="86" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="B86" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="G86" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H86" s="7"/>
+      <c r="I86" s="7"/>
+      <c r="J86" s="7"/>
+    </row>
+    <row r="87" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A87" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C87" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E87" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F87" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="G87" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="H87" s="7"/>
+      <c r="I87" s="7"/>
+      <c r="J87" s="7"/>
+    </row>
+    <row r="88" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A88" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B88" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G88" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="H88" s="7"/>
+      <c r="I88" s="7"/>
+      <c r="J88" s="7"/>
+    </row>
+    <row r="89" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A89" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="E89" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="F89" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="G89" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="H89" s="7"/>
+      <c r="I89" s="7"/>
+      <c r="J89" s="7"/>
+    </row>
+    <row r="90" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B90" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="G90" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="H90" s="7"/>
+      <c r="I90" s="7"/>
+      <c r="J90" s="7"/>
+    </row>
+    <row r="91" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A91" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D91" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E91" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="F91" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="G91" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="H91" s="7"/>
+      <c r="I91" s="7"/>
+      <c r="J91" s="7"/>
+    </row>
+    <row r="92" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="B92" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C92" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D92" s="7"/>
+      <c r="E92" s="7"/>
+      <c r="F92" s="7"/>
+      <c r="G92" s="7"/>
+      <c r="H92" s="7"/>
+      <c r="I92" s="7"/>
+      <c r="J92" s="7"/>
+    </row>
+    <row r="93" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A93" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="B93" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C93" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D93" s="7"/>
+      <c r="E93" s="7"/>
+      <c r="F93" s="7"/>
+      <c r="G93" s="7"/>
+      <c r="H93" s="7"/>
+      <c r="I93" s="7"/>
+      <c r="J93" s="7"/>
+    </row>
+    <row r="94" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A94" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C94" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D94" s="7"/>
+      <c r="E94" s="7"/>
+      <c r="F94" s="7"/>
+      <c r="G94" s="7"/>
+      <c r="H94" s="7"/>
+      <c r="I94" s="7"/>
+      <c r="J94" s="7"/>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A95" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C95" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D95" s="7"/>
+      <c r="E95" s="7"/>
+      <c r="F95" s="7"/>
+      <c r="G95" s="7"/>
+      <c r="H95" s="7"/>
+      <c r="I95" s="7"/>
+      <c r="J95" s="7"/>
+    </row>
+    <row r="96" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A96" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C96" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D96" s="7"/>
+      <c r="E96" s="7"/>
+      <c r="F96" s="7"/>
+      <c r="G96" s="7"/>
+      <c r="H96" s="7"/>
+      <c r="I96" s="7"/>
+      <c r="J96" s="7"/>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A97" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B97" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C97" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D97" s="7"/>
+      <c r="E97" s="7"/>
+      <c r="F97" s="7"/>
+      <c r="G97" s="7"/>
+      <c r="H97" s="7"/>
+      <c r="I97" s="7"/>
+      <c r="J97" s="7"/>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A98" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C98" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D98" s="7"/>
+      <c r="E98" s="7"/>
+      <c r="F98" s="7"/>
+      <c r="G98" s="7"/>
+      <c r="H98" s="7"/>
+      <c r="I98" s="7"/>
+      <c r="J98" s="7"/>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A99" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C99" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D99" s="7"/>
+      <c r="E99" s="7"/>
+      <c r="F99" s="7"/>
+      <c r="G99" s="7"/>
+      <c r="H99" s="7"/>
+      <c r="I99" s="7"/>
+      <c r="J99" s="7"/>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A100" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="B100" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C100" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D100" s="7"/>
+      <c r="E100" s="7"/>
+      <c r="F100" s="7"/>
+      <c r="G100" s="7"/>
+      <c r="H100" s="7"/>
+      <c r="I100" s="7"/>
+      <c r="J100" s="7"/>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A101" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B101" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C101" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D101" s="7"/>
+      <c r="E101" s="7"/>
+      <c r="F101" s="7"/>
+      <c r="G101" s="7"/>
+      <c r="H101" s="7"/>
+      <c r="I101" s="7"/>
+      <c r="J101" s="7"/>
+    </row>
+    <row r="102" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A102" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C102" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D102" s="7"/>
+      <c r="E102" s="7"/>
+      <c r="F102" s="7"/>
+      <c r="G102" s="7"/>
+      <c r="H102" s="7"/>
+      <c r="I102" s="7"/>
+      <c r="J102" s="7"/>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A103" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C103" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D103" s="7"/>
+      <c r="E103" s="7"/>
+      <c r="F103" s="7"/>
+      <c r="G103" s="7"/>
+      <c r="H103" s="7"/>
+      <c r="I103" s="7"/>
+      <c r="J103" s="7"/>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A104" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C104" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D104" s="7"/>
+      <c r="E104" s="7"/>
+      <c r="F104" s="7"/>
+      <c r="G104" s="7"/>
+      <c r="H104" s="7"/>
+      <c r="I104" s="7"/>
+      <c r="J104" s="7"/>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A105" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C105" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D105" s="7"/>
+      <c r="E105" s="7"/>
+      <c r="F105" s="7"/>
+      <c r="G105" s="7"/>
+      <c r="H105" s="7"/>
+      <c r="I105" s="7"/>
+      <c r="J105" s="7"/>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A106" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C106" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D106" s="7"/>
+      <c r="E106" s="7"/>
+      <c r="F106" s="7"/>
+      <c r="G106" s="7"/>
+      <c r="H106" s="7"/>
+      <c r="I106" s="7"/>
+      <c r="J106" s="7"/>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A107" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C107" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D107" s="7"/>
+      <c r="E107" s="7"/>
+      <c r="F107" s="7"/>
+      <c r="G107" s="7"/>
+      <c r="H107" s="7"/>
+      <c r="I107" s="7"/>
+      <c r="J107" s="7"/>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A108" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="B108" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C108" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D108" s="7"/>
+      <c r="E108" s="7"/>
+      <c r="F108" s="7"/>
+      <c r="G108" s="7"/>
+      <c r="H108" s="7"/>
+      <c r="I108" s="7"/>
+      <c r="J108" s="7"/>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A109" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C109" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D109" s="7"/>
+      <c r="E109" s="7"/>
+      <c r="F109" s="7"/>
+      <c r="G109" s="7"/>
+      <c r="H109" s="7"/>
+      <c r="I109" s="7"/>
+      <c r="J109" s="7"/>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A110" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C110" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D110" s="7"/>
+      <c r="E110" s="7"/>
+      <c r="F110" s="7"/>
+      <c r="G110" s="7"/>
+      <c r="H110" s="7"/>
+      <c r="I110" s="7"/>
+      <c r="J110" s="7"/>
+    </row>
+    <row r="111" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A111" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C111" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D111" s="7"/>
+      <c r="E111" s="7"/>
+      <c r="F111" s="7"/>
+      <c r="G111" s="7"/>
+      <c r="H111" s="7"/>
+      <c r="I111" s="7"/>
+      <c r="J111" s="7"/>
+    </row>
+    <row r="112" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A112" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C112" s="7"/>
+      <c r="D112" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E112" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="F112" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G112" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H112" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I112" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="J112" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A113" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C113" s="7"/>
+      <c r="D113" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G113" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="H113" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="I113" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="J113" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A114" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C114" s="7"/>
+      <c r="D114" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F114" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G114" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H114" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="I114" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="J114" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A115" s="9"/>
+      <c r="B115" s="8"/>
+      <c r="C115" s="8"/>
+      <c r="D115" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="G115" s="8"/>
+      <c r="H115" s="8"/>
+      <c r="I115" s="8"/>
+      <c r="J115" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A114:A115"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58CDA0BB-B524-4E22-9E95-FD736E9C2323}">
   <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1502,7 +3965,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>70</v>
       </c>
@@ -1543,7 +4006,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -1587,7 +4050,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -1631,7 +4094,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>93</v>
       </c>
@@ -1675,7 +4138,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="I15" s="2" t="s">
         <v>173</v>
       </c>
@@ -1695,7 +4158,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="I16" s="2" t="s">
         <v>179</v>
       </c>
@@ -1715,7 +4178,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="17" spans="9:14" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="9:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="I17" s="2" t="s">
         <v>185</v>
       </c>
@@ -1735,7 +4198,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="18" spans="9:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="9:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="I18" s="2" t="s">
         <v>191</v>
       </c>
@@ -1755,7 +4218,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="19" spans="9:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="9:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="I19" s="2" t="s">
         <v>197</v>
       </c>
@@ -1775,7 +4238,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="20" spans="9:14" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="9:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="I20" s="2" t="s">
         <v>202</v>
       </c>
@@ -1795,7 +4258,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="21" spans="9:14" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="9:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="I21" s="2" t="s">
         <v>208</v>
       </c>

</xml_diff>

<commit_message>
non-reproducable or non-deterministic shuffling
</commit_message>
<xml_diff>
--- a/Excel Files/OS.xlsx
+++ b/Excel Files/OS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub projects\Mcq_generator\Excel Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1EC09B-EE40-42E0-945F-3CD6A5B11949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8AC6F89-E036-4BA7-B888-EF2E0FED754B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A7744768-14E7-4F39-B6A5-4D54AC18E601}"/>
+    <workbookView xWindow="2040" yWindow="624" windowWidth="17280" windowHeight="9420" xr2:uid="{A7744768-14E7-4F39-B6A5-4D54AC18E601}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -875,7 +875,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -891,16 +891,106 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF92D050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3BEDFB"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3BEDFB"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC66FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3BEDFB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -908,11 +998,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -942,19 +1056,85 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -962,6 +1142,12 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF3BEDFB"/>
+      <color rgb="FFCC66FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1065,16 +1251,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>830580</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>381000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1055076</xdr:colOff>
+      <xdr:colOff>1032216</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>1249541</xdr:rowOff>
+      <xdr:rowOff>1630541</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1097,7 +1283,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2901462" y="18094569"/>
+          <a:off x="2872740" y="20124420"/>
           <a:ext cx="1055076" cy="1249541"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1508,7 +1694,7 @@
       </c>
     </row>
     <row r="3" spans="1:14" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="23" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -1517,13 +1703,13 @@
       <c r="D3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="30" t="s">
         <v>17</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="30" t="s">
         <v>19</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -1549,16 +1735,16 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="20" t="s">
         <v>24</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -1634,7 +1820,7 @@
       <c r="B6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="14" t="s">
         <v>36</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1713,7 +1899,7 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="22" t="s">
         <v>49</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -1804,7 +1990,7 @@
       <c r="D10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="12" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -1836,7 +2022,7 @@
       </c>
     </row>
     <row r="11" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="21" t="s">
         <v>70</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1877,10 +2063,10 @@
       </c>
     </row>
     <row r="12" spans="1:14" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="28" t="s">
         <v>78</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1892,10 +2078,10 @@
       <c r="E12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="28" t="s">
         <v>83</v>
       </c>
       <c r="H12" s="2" t="s">
@@ -1921,11 +2107,11 @@
       </c>
     </row>
     <row r="13" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12" t="s">
+      <c r="A13" s="26"/>
+      <c r="B13" s="27" t="s">
         <v>249</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="29" t="s">
         <v>250</v>
       </c>
       <c r="D13" s="9" t="s">
@@ -1965,7 +2151,7 @@
       <c r="C14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="22" t="s">
         <v>86</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -2006,7 +2192,7 @@
       <c r="D15" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="15" t="s">
         <v>265</v>
       </c>
       <c r="F15" s="2"/>
@@ -2040,7 +2226,7 @@
       <c r="D16" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="14" t="s">
         <v>264</v>
       </c>
       <c r="F16" s="2"/>
@@ -2066,13 +2252,13 @@
       </c>
     </row>
     <row r="17" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="31" t="s">
         <v>256</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="18" t="s">
         <v>92</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -2110,14 +2296,14 @@
       </c>
     </row>
     <row r="18" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="11"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="32"/>
+      <c r="B18" s="33" t="s">
         <v>245</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="16" t="s">
         <v>246</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="35" t="s">
         <v>248</v>
       </c>
       <c r="I18" s="2" t="s">
@@ -2140,13 +2326,13 @@
       </c>
     </row>
     <row r="19" spans="1:14" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="36" t="s">
         <v>260</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="19" t="s">
         <v>266</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="10" t="s">
         <v>261</v>
       </c>
       <c r="I19" s="2" t="s">
@@ -2169,7 +2355,7 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="24" t="s">
         <v>262</v>
       </c>
       <c r="I20" s="2" t="s">
@@ -2192,7 +2378,7 @@
       </c>
     </row>
     <row r="21" spans="1:14" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="34" t="s">
         <v>263</v>
       </c>
       <c r="I21" s="2" t="s">
@@ -2215,7 +2401,7 @@
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="E22" s="12"/>
+      <c r="E22" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4493,7 +4679,7 @@
       </c>
     </row>
     <row r="114" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A114" s="10" t="s">
+      <c r="A114" s="11" t="s">
         <v>244</v>
       </c>
       <c r="B114" s="8" t="s">
@@ -4523,7 +4709,7 @@
       </c>
     </row>
     <row r="115" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A115" s="10"/>
+      <c r="A115" s="11"/>
       <c r="B115" s="8"/>
       <c r="C115" s="8"/>
       <c r="D115" s="8" t="s">

</xml_diff>